<commit_message>
Sync review data 2026-10-20
</commit_message>
<xml_diff>
--- a/review-results/复盘信息抓取-20261020.xlsx
+++ b/review-results/复盘信息抓取-20261020.xlsx
@@ -5113,148 +5113,1060 @@
       </c>
     </row>
     <row r="2">
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>12791.307</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>192.42</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>828.278</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>461.8</v>
+      </c>
     </row>
     <row r="3">
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>12883.761</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>216.315</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>737.322</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>260.61</v>
+      </c>
     </row>
     <row r="4">
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>14616.199</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>344.908</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>821.612</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>461.8</v>
+      </c>
     </row>
     <row r="5">
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>13892.348</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>396.175</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>837.143</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>461.8</v>
+      </c>
     </row>
     <row r="6">
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>13828.187</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>430.688</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>891.217</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>472.19</v>
+      </c>
     </row>
     <row r="7">
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>13910.498</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>465.52</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>882.1420000000001</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>472.19</v>
+      </c>
     </row>
     <row r="8">
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>14686.735</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>440.13</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>1055.385</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>487.42</v>
+      </c>
     </row>
     <row r="9">
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>14331.453</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>293.5</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>725.408</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>260.61</v>
+      </c>
     </row>
     <row r="10">
-      <c r="D10" s="3" t="n"/>
-      <c r="E10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>12992.783</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>281.058</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>09</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>215.513</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>103.59</v>
+      </c>
     </row>
     <row r="11">
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>11840.559</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>85.658</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>180.936</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>13632.87</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>127.395</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>71.495</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
-      <c r="L13" s="3" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>15763.63</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>300.275</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>72.34699999999999</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
-      <c r="L14" s="3" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>16641.725</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>380.563</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>72.833</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
-      <c r="L15" s="3" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>17875.84</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>300.153</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>114.288</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>107.52</v>
+      </c>
     </row>
     <row r="16">
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>16706.283</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>238.918</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>203.882</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>107.52</v>
+      </c>
     </row>
     <row r="17">
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
-      <c r="L17" s="3" t="n"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>15505.631</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>438.228</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>358.774</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>348.89</v>
+      </c>
     </row>
     <row r="18">
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
-      <c r="L18" s="3" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>15059.538</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>472.68</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>856.797</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>470.86</v>
+      </c>
     </row>
     <row r="19">
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
-      <c r="L19" s="3" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>14952.734</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>476.69</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>973.807</v>
+      </c>
+      <c r="L19" s="3" t="n">
+        <v>486.51</v>
+      </c>
     </row>
     <row r="20">
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
-      <c r="L20" s="3" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>13569.114</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>337.9</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>797.0069999999999</v>
+      </c>
+      <c r="L20" s="3" t="n">
+        <v>462.63</v>
+      </c>
     </row>
     <row r="21">
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
-      <c r="L21" s="3" t="n"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>13200.032</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>335.305</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>759.515</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>430.8</v>
+      </c>
     </row>
     <row r="22">
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>14868.147</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>367.658</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>789.112</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>461.8</v>
+      </c>
     </row>
     <row r="23">
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
-      <c r="L23" s="3" t="n"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>15302.28</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>209.418</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>725.982</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>430.66</v>
+      </c>
     </row>
     <row r="24">
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
-      <c r="L24" s="3" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>14272.033</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>91.19499999999999</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>700.1369999999999</v>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>259.5</v>
+      </c>
     </row>
     <row r="25">
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
-      <c r="L25" s="3" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>现货实时交易价格曲线</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>14163.96</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>118.698</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>现货日前交易价格曲线</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>694.196</v>
+      </c>
+      <c r="L25" s="3" t="n">
+        <v>259.5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16375,24 +17287,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>非市场化机组总出力</t>
+          <t>现货实时交易价格曲线</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>96</v>
+        <v>24</v>
       </c>
       <c r="C2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>新能源实际发电曲线</t>
+          <t>现货日前交易价格曲线</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>96</v>
+        <v>24</v>
       </c>
       <c r="C3" t="n">
         <v>5</v>
@@ -16401,7 +17313,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>实际系统负荷</t>
+          <t>非市场化机组总出力</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -16414,70 +17326,94 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>省间联络线输电情况</t>
+          <t>新能源实际发电曲线</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>96</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>各时段各类电源电量</t>
+          <t>实际系统负荷</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>960</v>
+        <v>96</v>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>各时段各类电源的开机台数</t>
+          <t>省间联络线输电情况</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>768</v>
+        <v>96</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>实时储能充电计划及电价</t>
+          <t>各时段各类电源电量</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>96</v>
+        <v>960</v>
       </c>
       <c r="C8" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>各时段各类电源的开机台数</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>768</v>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>实时储能充电计划及电价</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>96</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>日前储能充电计划及电价</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B11" t="n">
         <v>96</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C11" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>